<commit_message>
Update expected prediction data in Excel file
</commit_message>
<xml_diff>
--- a/APP/modelo_previsao/dados_previsao_esperados.xlsx
+++ b/APP/modelo_previsao/dados_previsao_esperados.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b96299a9c75324a7/Área de Trabalho/Enterprise Challenge/APP/modelo_previsao/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B113A31C-E4BB-46C6-ADF1-E7A316ECCFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{B113A31C-E4BB-46C6-ADF1-E7A316ECCFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A8143A7-AD23-4CE3-9F55-75E17371482F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0523AF9C-A823-4FC6-B10E-CA9FA3EB788C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{0523AF9C-A823-4FC6-B10E-CA9FA3EB788C}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -319,7 +319,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -336,13 +336,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -353,9 +352,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -701,109 +697,107 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EEDB2C1-998B-4DBC-A2C0-22DAEDCC391A}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="17.7109375" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5703125" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.7109375" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="9" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="13" t="s">
+      <c r="I1" s="10"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="L1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="N2" s="15"/>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15"/>
-      <c r="Q2" s="16"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="14"/>
     </row>
-    <row r="3" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
+    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="N2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="O2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="P2" s="6" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="M2:Q2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="L1:P1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>